<commit_message>
Small typo fixed in RiskRegister.xlsx
</commit_message>
<xml_diff>
--- a/docs/05-risk-assurance/RiskRegister.xlsx
+++ b/docs/05-risk-assurance/RiskRegister.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\git\ml-production-assurance-framework\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\git\ai-ml-engineering-framework\docs\05-risk-assurance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A3D5C55-543D-46A4-9701-60F46063DE2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241E743A-39B7-469F-A668-EA8E4441E4BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,9 +55,6 @@
     <t>Risk Grade</t>
   </si>
   <si>
-    <t>Quantified Risk Lilelihood</t>
-  </si>
-  <si>
     <t>Quantified Risk Impact</t>
   </si>
   <si>
@@ -77,6 +74,9 @@
   </si>
   <si>
     <t>Risk register structure adapted from standard project risk management frameworks used in teaching and industry practice.</t>
+  </si>
+  <si>
+    <t>Quantified Risk Likelihood</t>
   </si>
 </sst>
 </file>
@@ -408,25 +408,25 @@
         <v>10</v>
       </c>
       <c r="L1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>17</v>
       </c>
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
@@ -439,7 +439,7 @@
     </row>
     <row r="32" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add V&V plan and verification/validation register
</commit_message>
<xml_diff>
--- a/docs/05-risk-assurance/RiskRegister.xlsx
+++ b/docs/05-risk-assurance/RiskRegister.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\git\ai-ml-engineering-framework\docs\05-risk-assurance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241E743A-39B7-469F-A668-EA8E4441E4BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA6D309A-5848-4DCF-A548-8CE0F6B95225}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>ID</t>
   </si>
@@ -77,13 +77,28 @@
   </si>
   <si>
     <t>Quantified Risk Likelihood</t>
+  </si>
+  <si>
+    <t>RISK-001</t>
+  </si>
+  <si>
+    <t>RISK-002</t>
+  </si>
+  <si>
+    <t>RISK-003</t>
+  </si>
+  <si>
+    <t>RISK-004</t>
+  </si>
+  <si>
+    <t>RISK-005</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -94,12 +109,21 @@
       <sz val="16"/>
       <color theme="0"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="16"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13.5"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -129,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -138,6 +162,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -359,6 +384,7 @@
   <dimension ref="A1:Z32"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="14.28515625" customWidth="1"/>
     <col min="2" max="2" width="17.42578125" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="14.42578125" customWidth="1"/>
@@ -437,6 +463,31 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
+    <row r="2" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
     <row r="32" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
Added Benefits Register - useful for project advocacy
</commit_message>
<xml_diff>
--- a/docs/05-risk-assurance/RiskRegister.xlsx
+++ b/docs/05-risk-assurance/RiskRegister.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\git\ai-ml-engineering-framework\docs\05-risk-assurance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA6D309A-5848-4DCF-A548-8CE0F6B95225}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3220C024-7AB6-4785-9AFB-9346C762290D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="RISK" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -381,7 +381,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z32"/>
+  <dimension ref="A1:R32"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.28515625" customWidth="1"/>
@@ -399,7 +399,7 @@
     <col min="18" max="18" width="17.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -454,36 +454,28 @@
       <c r="R1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-      <c r="W1" s="1"/>
-      <c r="X1" s="1"/>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="1"/>
-    </row>
-    <row r="2" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>23</v>
       </c>

</xml_diff>